<commit_message>
submit income per capita
</commit_message>
<xml_diff>
--- a/SType3.xlsx
+++ b/SType3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy-GGP-Sumsel-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{0EE31145-1C28-4746-9AD6-ACD75441FBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{14669CFE-8272-4C38-920D-82EE542AB5C7}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{0EE31145-1C28-4746-9AD6-ACD75441FBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48750D07-8F6F-4327-9A51-43D942EA0B05}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EC239BBC-85AB-4F2B-8A61-BB5BEF637A63}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EC239BBC-85AB-4F2B-8A61-BB5BEF637A63}"/>
   </bookViews>
   <sheets>
     <sheet name="SType3" sheetId="1" r:id="rId1"/>
@@ -417,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A73147C-AEBD-440B-8DAA-C77F4C7A39D8}">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
@@ -562,6 +562,148 @@
         <v>0.89999999999999991</v>
       </c>
     </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>9.9999999999999978E-2</v>
+      </c>
+      <c r="F3">
+        <v>0.14444444444444443</v>
+      </c>
+      <c r="G3">
+        <v>0.18888888888888886</v>
+      </c>
+      <c r="H3">
+        <v>0.23333333333333331</v>
+      </c>
+      <c r="I3">
+        <v>0.27777777777777779</v>
+      </c>
+      <c r="J3">
+        <v>0.32222222222222219</v>
+      </c>
+      <c r="K3">
+        <v>0.36666666666666664</v>
+      </c>
+      <c r="L3">
+        <v>0.41111111111111109</v>
+      </c>
+      <c r="M3">
+        <v>0.45555555555555555</v>
+      </c>
+      <c r="N3">
+        <v>0.5</v>
+      </c>
+      <c r="O3">
+        <v>0.54444444444444451</v>
+      </c>
+      <c r="P3">
+        <v>0.5888888888888888</v>
+      </c>
+      <c r="Q3">
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="R3">
+        <v>0.67777777777777781</v>
+      </c>
+      <c r="S3">
+        <v>0.72222222222222232</v>
+      </c>
+      <c r="T3">
+        <v>0.76666666666666661</v>
+      </c>
+      <c r="U3">
+        <v>0.81111111111111112</v>
+      </c>
+      <c r="V3">
+        <v>0.85555555555555562</v>
+      </c>
+      <c r="W3">
+        <v>0.89999999999999991</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>19</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>9.9999999999999978E-2</v>
+      </c>
+      <c r="F4">
+        <v>0.14444444444444443</v>
+      </c>
+      <c r="G4">
+        <v>0.18888888888888886</v>
+      </c>
+      <c r="H4">
+        <v>0.23333333333333331</v>
+      </c>
+      <c r="I4">
+        <v>0.27777777777777779</v>
+      </c>
+      <c r="J4">
+        <v>0.32222222222222219</v>
+      </c>
+      <c r="K4">
+        <v>0.36666666666666664</v>
+      </c>
+      <c r="L4">
+        <v>0.41111111111111109</v>
+      </c>
+      <c r="M4">
+        <v>0.45555555555555555</v>
+      </c>
+      <c r="N4">
+        <v>0.5</v>
+      </c>
+      <c r="O4">
+        <v>0.54444444444444451</v>
+      </c>
+      <c r="P4">
+        <v>0.5888888888888888</v>
+      </c>
+      <c r="Q4">
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="R4">
+        <v>0.67777777777777781</v>
+      </c>
+      <c r="S4">
+        <v>0.72222222222222232</v>
+      </c>
+      <c r="T4">
+        <v>0.76666666666666661</v>
+      </c>
+      <c r="U4">
+        <v>0.81111111111111112</v>
+      </c>
+      <c r="V4">
+        <v>0.85555555555555562</v>
+      </c>
+      <c r="W4">
+        <v>0.89999999999999991</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update Stype3 dan Stype 1
</commit_message>
<xml_diff>
--- a/SType3.xlsx
+++ b/SType3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy-GGP-Sumsel-2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{0EE31145-1C28-4746-9AD6-ACD75441FBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8643FFD2-2650-4A70-AC7C-A75020A2E888}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{0EE31145-1C28-4746-9AD6-ACD75441FBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E15DD00-2964-44B9-ABA3-3B635EB87A01}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EC239BBC-85AB-4F2B-8A61-BB5BEF637A63}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{EC239BBC-85AB-4F2B-8A61-BB5BEF637A63}"/>
   </bookViews>
   <sheets>
     <sheet name="SType3" sheetId="1" r:id="rId1"/>
@@ -420,7 +420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A73147C-AEBD-440B-8DAA-C77F4C7A39D8}">
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
@@ -736,208 +736,60 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>9.9999999999999978E-2</v>
       </c>
       <c r="G5">
-        <v>0.10000000000000003</v>
+        <v>0.14444444444444443</v>
       </c>
       <c r="H5">
-        <v>0.1470588235294118</v>
+        <v>0.18888888888888886</v>
       </c>
       <c r="I5">
-        <v>0.19411764705882353</v>
+        <v>0.23333333333333331</v>
       </c>
       <c r="J5">
-        <v>0.2411764705882353</v>
+        <v>0.27777777777777779</v>
       </c>
       <c r="K5">
-        <v>0.28823529411764703</v>
+        <v>0.32222222222222219</v>
       </c>
       <c r="L5">
-        <v>0.3352941176470588</v>
+        <v>0.36666666666666664</v>
       </c>
       <c r="M5">
-        <v>0.38235294117647056</v>
+        <v>0.41111111111111109</v>
       </c>
       <c r="N5">
-        <v>0.42941176470588233</v>
+        <v>0.45555555555555555</v>
       </c>
       <c r="O5">
-        <v>0.47647058823529409</v>
+        <v>0.5</v>
       </c>
       <c r="P5">
-        <v>0.5235294117647058</v>
+        <v>0.54444444444444451</v>
       </c>
       <c r="Q5">
-        <v>0.57058823529411762</v>
+        <v>0.5888888888888888</v>
       </c>
       <c r="R5">
-        <v>0.61764705882352933</v>
+        <v>0.6333333333333333</v>
       </c>
       <c r="S5">
-        <v>0.66470588235294115</v>
+        <v>0.67777777777777781</v>
       </c>
       <c r="T5">
-        <v>0.71176470588235285</v>
+        <v>0.72222222222222232</v>
       </c>
       <c r="U5">
-        <v>0.75882352941176467</v>
+        <v>0.76666666666666661</v>
       </c>
       <c r="V5">
-        <v>0.80588235294117638</v>
+        <v>0.81111111111111112</v>
       </c>
       <c r="W5">
-        <v>0.85294117647058809</v>
+        <v>0.85555555555555562</v>
       </c>
       <c r="X5">
-        <v>0.89999999999999991</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>302</v>
-      </c>
-      <c r="B6">
-        <v>51</v>
-      </c>
-      <c r="C6">
-        <v>33</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0.10000000000000003</v>
-      </c>
-      <c r="H6">
-        <v>0.1470588235294118</v>
-      </c>
-      <c r="I6">
-        <v>0.19411764705882353</v>
-      </c>
-      <c r="J6">
-        <v>0.2411764705882353</v>
-      </c>
-      <c r="K6">
-        <v>0.28823529411764703</v>
-      </c>
-      <c r="L6">
-        <v>0.3352941176470588</v>
-      </c>
-      <c r="M6">
-        <v>0.38235294117647056</v>
-      </c>
-      <c r="N6">
-        <v>0.42941176470588233</v>
-      </c>
-      <c r="O6">
-        <v>0.47647058823529409</v>
-      </c>
-      <c r="P6">
-        <v>0.5235294117647058</v>
-      </c>
-      <c r="Q6">
-        <v>0.57058823529411762</v>
-      </c>
-      <c r="R6">
-        <v>0.61764705882352933</v>
-      </c>
-      <c r="S6">
-        <v>0.66470588235294115</v>
-      </c>
-      <c r="T6">
-        <v>0.71176470588235285</v>
-      </c>
-      <c r="U6">
-        <v>0.75882352941176467</v>
-      </c>
-      <c r="V6">
-        <v>0.80588235294117638</v>
-      </c>
-      <c r="W6">
-        <v>0.85294117647058809</v>
-      </c>
-      <c r="X6">
-        <v>0.89999999999999991</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>302</v>
-      </c>
-      <c r="B7">
-        <v>51</v>
-      </c>
-      <c r="C7">
-        <v>37</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0.10000000000000003</v>
-      </c>
-      <c r="H7">
-        <v>0.1470588235294118</v>
-      </c>
-      <c r="I7">
-        <v>0.19411764705882353</v>
-      </c>
-      <c r="J7">
-        <v>0.2411764705882353</v>
-      </c>
-      <c r="K7">
-        <v>0.28823529411764703</v>
-      </c>
-      <c r="L7">
-        <v>0.3352941176470588</v>
-      </c>
-      <c r="M7">
-        <v>0.38235294117647056</v>
-      </c>
-      <c r="N7">
-        <v>0.42941176470588233</v>
-      </c>
-      <c r="O7">
-        <v>0.47647058823529409</v>
-      </c>
-      <c r="P7">
-        <v>0.5235294117647058</v>
-      </c>
-      <c r="Q7">
-        <v>0.57058823529411762</v>
-      </c>
-      <c r="R7">
-        <v>0.61764705882352933</v>
-      </c>
-      <c r="S7">
-        <v>0.66470588235294115</v>
-      </c>
-      <c r="T7">
-        <v>0.71176470588235285</v>
-      </c>
-      <c r="U7">
-        <v>0.75882352941176467</v>
-      </c>
-      <c r="V7">
-        <v>0.80588235294117638</v>
-      </c>
-      <c r="W7">
-        <v>0.85294117647058809</v>
-      </c>
-      <c r="X7">
         <v>0.89999999999999991</v>
       </c>
     </row>

</xml_diff>